<commit_message>
Koreksi klaim formula (3.300+, akurat) + refresh unduhan gratis
</commit_message>
<xml_diff>
--- a/downloads/GRATIS - Pembukuan Kas UMKM.xlsx
+++ b/downloads/GRATIS - Pembukuan Kas UMKM.xlsx
@@ -996,7 +996,7 @@
   <sheetPr>
     <tabColor rgb="000F766E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -2634,6 +2634,8 @@
       <formula1>36526</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>